<commit_message>
checklist artefato 4 preenchido
</commit_message>
<xml_diff>
--- a/Checklist - Artefato 2.xlsx
+++ b/Checklist - Artefato 2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rafael Fernandes\Downloads\ChecklistQualidade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACC326C9-D6D8-4D3F-93F2-C82861A2BD7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC8D7DDD-EC4D-4103-BE89-B853C42A8EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -337,24 +337,24 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -961,16 +961,16 @@
       <c r="H21" s="5"/>
     </row>
     <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="10" t="s">
         <v>28</v>
       </c>
       <c r="C25" s="8"/>
-      <c r="E25" s="9" t="s">
+      <c r="E25" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="F25" s="9"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="9"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11"/>
+      <c r="H25" s="11"/>
     </row>
     <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="6" t="s">
@@ -979,16 +979,16 @@
       <c r="C26" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="F26" s="11" t="s">
+      <c r="F26" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="H26" s="11" t="s">
+      <c r="H26" s="14" t="s">
         <v>43</v>
       </c>
     </row>
@@ -999,10 +999,10 @@
       <c r="C27" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="E27" s="12"/>
-      <c r="F27" s="13"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="15"/>
     </row>
     <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="6" t="s">
@@ -1011,16 +1011,16 @@
       <c r="C28" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="E28" s="14">
+      <c r="E28" s="9">
         <v>0</v>
       </c>
-      <c r="F28" s="14">
+      <c r="F28" s="9">
         <v>0</v>
       </c>
-      <c r="G28" s="14">
+      <c r="G28" s="9">
         <v>0</v>
       </c>
-      <c r="H28" s="14">
+      <c r="H28" s="9">
         <v>0</v>
       </c>
     </row>
@@ -1073,6 +1073,14 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="aed73f09-bf5d-4147-a3d9-eca4840d3416" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101007CCF20922A0DE34DA3357EDA40AE3850" ma:contentTypeVersion="5" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="df2c289d3a08b18055ba2ef47a57998b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="aed73f09-bf5d-4147-a3d9-eca4840d3416" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="91dac5f1c2bd6141b57005fd2a16424c" ns3:_="">
     <xsd:import namespace="aed73f09-bf5d-4147-a3d9-eca4840d3416"/>
@@ -1222,14 +1230,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="aed73f09-bf5d-4147-a3d9-eca4840d3416" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{398CE32A-8B97-402C-8C2F-6E1932019FB4}">
   <ds:schemaRefs>
@@ -1239,6 +1239,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F272DB39-8BAE-464A-AAA3-19537EA33ACE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="aed73f09-bf5d-4147-a3d9-eca4840d3416"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F3887D1-A29C-405D-BB37-6D7E8E326CC9}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1254,20 +1270,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F272DB39-8BAE-464A-AAA3-19537EA33ACE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="aed73f09-bf5d-4147-a3d9-eca4840d3416"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>